<commit_message>
§10 clear cases (Lysozincrosis SUBTYPE/L2, Aponecrosis UMBRELLA, Pyronecrosis SYNONYM) + L5 rename (drop legacy/emerging)
</commit_message>
<xml_diff>
--- a/app/data/RCDome_Decoder_53.xlsx
+++ b/app/data/RCDome_Decoder_53.xlsx
@@ -1176,7 +1176,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LEGACY</t>
+          <t>UMBRELLA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1321,7 +1321,12 @@
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>associated_with</t>
+          <t>umbrella_for</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>Apoptosis; Necrosis</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
@@ -4841,7 +4846,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>LEGACY</t>
+          <t>SUBTYPE</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -4856,7 +4861,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>A lysosome-dependent cell-death process (legacy term) demarcated by lysosomal membrane permeabilization and cathepsin-dependent cytoplasmic proteolysis, executed when serpin inhibition is absent.</t>
+          <t>A lysosome-dependent cell-death subtype demarcated by serpin/SERPINB3-moderated lysosomal membrane permeabilization and cathepsin-L-dependent cytoplasmic proteolysis, executed in the absence of neutralizing endogenous serpin inhibition.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -4981,7 +4986,7 @@
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>supported</t>
         </is>
       </c>
       <c r="AI25" t="inlineStr">
@@ -5397,7 +5402,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EMERGING</t>
+          <t>SUBTYPE</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -5547,7 +5552,7 @@
       </c>
       <c r="AI28" t="inlineStr">
         <is>
-          <t>associated_with</t>
+          <t>subtype_of</t>
         </is>
       </c>
       <c r="AJ28" t="inlineStr">
@@ -9057,7 +9062,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>LEGACY</t>
+          <t>SYNONYM</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -9202,7 +9207,7 @@
       </c>
       <c r="AI48" t="inlineStr">
         <is>
-          <t>associated_with</t>
+          <t>synonym_of</t>
         </is>
       </c>
       <c r="AJ48" t="inlineStr">

</xml_diff>

<commit_message>
§10 deferred: Floatptosis + Spectosis -> CELL_TYPE (L4); fix figure-legend L5 name + restore ¶383 formatting
</commit_message>
<xml_diff>
--- a/app/data/RCDome_Decoder_53.xlsx
+++ b/app/data/RCDome_Decoder_53.xlsx
@@ -4148,7 +4148,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>EMERGING</t>
+          <t>CELL_TYPE</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -9775,7 +9775,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>EMERGING</t>
+          <t>CELL_TYPE</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">

</xml_diff>

<commit_message>
§8/§10: NECSO -> CORE_PENDING / L1-ELIGIBLE (emerging) — G1+G2 passed (TRPM4 KO resistance + inhibitors); proportions L1 17, L5 14
</commit_message>
<xml_diff>
--- a/app/data/RCDome_Decoder_53.xlsx
+++ b/app/data/RCDome_Decoder_53.xlsx
@@ -7429,12 +7429,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>LEGACY</t>
+          <t>CORE_PENDING</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>NOT-L1</t>
+          <t>L1-ELIGIBLE</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -7444,7 +7444,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>A necrotic cell-death process (legacy term) caused by sodium overload, executed via persistent activation of the TRPM4 cation channel by necrocide 1.</t>
+          <t>A necrotic cell-death modality caused by sodium overload, executed via persistent activation of the TRPM4 cation channel by necrocide 1 (NC1).</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -7544,7 +7544,7 @@
       </c>
       <c r="AC39" t="inlineStr">
         <is>
-          <t>Retain source label unchanged pending expansion and definition.</t>
+          <t>Candidate modality (G1+G2 passed); G5 replication pending; human TRPM4-specific.</t>
         </is>
       </c>
       <c r="AD39" t="inlineStr">
@@ -7569,7 +7569,7 @@
       </c>
       <c r="AH39" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>emerging</t>
         </is>
       </c>
       <c r="AI39" t="inlineStr">

</xml_diff>

<commit_message>
§10: Mitoxyperilysis -> CORE_PENDING / L1-ELIGIBLE (emerging) — full-text G2 KO evidence (Bax/Bak1/Bid triple-KO, PMC12875127); proportions L1 18, L5 13
</commit_message>
<xml_diff>
--- a/app/data/RCDome_Decoder_53.xlsx
+++ b/app/data/RCDome_Decoder_53.xlsx
@@ -6681,12 +6681,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>EMERGING</t>
+          <t>CORE_PENDING</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>NOT-L1</t>
+          <t>L1-ELIGIBLE</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -6696,7 +6696,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>A lytic cell-death process (emerging concept) triggered by the synergism of innate-immune and metabolic signals, demarcated by BAX/BAK1/BID-dependent mitochondrial oxidative stress at the plasma membrane and culminating in membrane lysis.</t>
+          <t>A lytic cell-death modality triggered by the synergism of innate-immune and metabolic signals, demarcated by BAX/BAK1/BID-dependent mitochondrial oxidative stress at the plasma membrane and culminating in membrane lysis.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -6796,7 +6796,7 @@
       </c>
       <c r="AC35" t="inlineStr">
         <is>
-          <t>Retain as supplied pending a frozen operational definition.</t>
+          <t>Candidate modality (G1+G2 passed; G2 by CRISPR/Cas9 Bax/Bak1/Bid triple-KO resistance, PMC12875127; distinct from MPT (CsA/CypD) and NLRP3); G5 replication pending; human.</t>
         </is>
       </c>
       <c r="AD35" t="inlineStr">

</xml_diff>

<commit_message>
Propagate Triaptosis founding PMID 39638924->39446948 to builder, S3/S12, D1, consensus report
</commit_message>
<xml_diff>
--- a/app/data/RCDome_Decoder_53.xlsx
+++ b/app/data/RCDome_Decoder_53.xlsx
@@ -9947,12 +9947,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>EMERGING</t>
+          <t>CORE_PENDING</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>NOT-L1</t>
+          <t>L1-ELIGIBLE</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -9962,7 +9962,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>An endosome-dependent cell-death process (emerging concept).</t>
+          <t>An endosome-dependent cell-death modality executed through VPS34/PIK3C3 inhibition (oxidation of Cys54/Cys61) and endosomal-identity loss.</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -9972,7 +9972,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>39638924</t>
+          <t>39446948</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -9982,7 +9982,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>39638924</t>
+          <t>39446948;39638924</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -10037,7 +10037,7 @@
       </c>
       <c r="W53" t="inlineStr">
         <is>
-          <t>39638924</t>
+          <t>39446948</t>
         </is>
       </c>
       <c r="X53" t="inlineStr">
@@ -10062,7 +10062,7 @@
       </c>
       <c r="AC53" t="inlineStr">
         <is>
-          <t>Retain as supplied pending a frozen operational definition.</t>
+          <t>Candidate modality (G1+G2 passed; G2 by VPS34 CRISPR-KO + WT-rescue + Cys54/61 non-rescue, PMC11975464); G5 replication pending; human + mouse.</t>
         </is>
       </c>
       <c r="AD53" t="inlineStr">

</xml_diff>

<commit_message>
§3/§4 rename: Entosis->Entotic cell death, NETosis->NETotic cell death (canonical); process names preserved as source strings; manuscript ¶54/90 updated
</commit_message>
<xml_diff>
--- a/app/data/RCDome_Decoder_53.xlsx
+++ b/app/data/RCDome_Decoder_53.xlsx
@@ -3410,7 +3410,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Entosis</t>
+          <t>Entotic cell death</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3550,7 +3550,7 @@
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>Use entotic cell death as the canonical concept name. [2]</t>
+          <t>Entotic cell death (death) originating from entosis (cell-in-cell process); entosis is the source/process term.</t>
         </is>
       </c>
       <c r="AD17" t="inlineStr">
@@ -7596,7 +7596,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>NETosis</t>
+          <t>NETotic cell death</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7736,7 +7736,7 @@
       </c>
       <c r="AC40" t="inlineStr">
         <is>
-          <t>Retain as a distinct regulated-necrosis modality. [2, 4]</t>
+          <t>NETotic cell death (death) associated with NETosis (NET-release process); NETosis is the source/process term.</t>
         </is>
       </c>
       <c r="AD40" t="inlineStr">

</xml_diff>

<commit_message>
Nomenclature harmonization: C1-C5->MC1-MC5, C1-C6->RS1-RS6, Q1-Q5->QG1-QG5, T1-T4->ET1-ET4/CT1-CT4 (crosswalk + decoder/matrix/tables/manuscript/app) + fix 16/53->19/53
</commit_message>
<xml_diff>
--- a/app/data/RCDome_Decoder_53.xlsx
+++ b/app/data/RCDome_Decoder_53.xlsx
@@ -493,32 +493,32 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>RS1</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>RS2</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>RS3</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>RS4</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>RS5</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>RS6</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">

</xml_diff>